<commit_message>
Fix issue in remaining items
</commit_message>
<xml_diff>
--- a/public/manifest/sample_price_manifest.xlsx
+++ b/public/manifest/sample_price_manifest.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6189" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6186" uniqueCount="99">
   <si>
     <t>CBX</t>
   </si>
@@ -313,15 +313,6 @@
   </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>arrival_price</t>
-  </si>
-  <si>
-    <t>departure_price</t>
-  </si>
-  <si>
-    <t>round_trip_price</t>
   </si>
 </sst>
 </file>
@@ -842,15 +833,9 @@
       <c r="I1" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="J1" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="K1" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="L1" s="15" t="s">
-        <v>101</v>
-      </c>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>

</xml_diff>